<commit_message>
add some settings, fix backend
</commit_message>
<xml_diff>
--- a/backend/resource/templates/template.xlsx
+++ b/backend/resource/templates/template.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B4A53BD-31C5-4FBE-80E7-7F6D2006709B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E7C30DE-AD67-4BFA-AFFD-09F9DB2A5169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3420" yWindow="3420" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4110" yWindow="4110" windowWidth="21600" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Смета" sheetId="1" r:id="rId1"/>
@@ -617,8 +617,8 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.28515625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="68.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="8.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="65.42578125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" style="2" customWidth="1"/>
     <col min="4" max="4" width="9.85546875" style="8" customWidth="1"/>
     <col min="5" max="5" width="10.7109375" style="8" customWidth="1"/>
     <col min="6" max="6" width="14.28515625" style="9" customWidth="1"/>
@@ -726,6 +726,6 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="85" fitToHeight="2" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="86" fitToHeight="2" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>